<commit_message>
Fix dashboard zeros by removing N-column formula chain
Replace intermediate liaison column (N) with direct cross-sheet cell
references in the Tableau de Bord. openpyxl stores formula cells with
cached value=0; by pointing directly at intra-sheet cells (B3, B4, F10,
H10…) the formulas resolve correctly in Excel and Google Sheets.
Also add fullCalcOnLoad=True to force recalculation on file open.

https://claude.ai/code/session_011YmAwaQupv4S7DU5Q3eXc2
</commit_message>
<xml_diff>
--- a/Comptabilite_Fournisseur.xlsx
+++ b/Comptabilite_Fournisseur.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Op. Agro-alimentaire" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="#,##0 &quot;F&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,11 +54,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00595959"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00595959"/>
       <sz val="10"/>
@@ -80,11 +75,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -158,15 +148,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -193,19 +183,19 @@
     <xf numFmtId="165" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -220,7 +210,6 @@
     <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -230,7 +219,6 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -240,13 +228,13 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -699,27 +687,27 @@
         </is>
       </c>
       <c r="C4" s="6">
-        <f>'Op. Poisson Séché'!N4</f>
+        <f>'Op. Poisson Séché'!B3</f>
         <v/>
       </c>
       <c r="D4" s="6">
-        <f>'Op. Poisson Séché'!N6</f>
+        <f>'Op. Poisson Séché'!B4</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>'Op. Poisson Séché'!N8</f>
+        <f>'Op. Poisson Séché'!B5</f>
         <v/>
       </c>
       <c r="F4" s="6">
-        <f>'Op. Poisson Séché'!N10</f>
+        <f>'Op. Poisson Séché'!B9</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>'Op. Poisson Séché'!N12</f>
+        <f>'Op. Poisson Séché'!B8</f>
         <v/>
       </c>
       <c r="H4" s="7">
-        <f>'Op. Poisson Séché'!N13</f>
+        <f>'Op. Poisson Séché'!B10</f>
         <v/>
       </c>
     </row>
@@ -733,32 +721,32 @@
         </is>
       </c>
       <c r="C5" s="10">
-        <f>'Op. Agro-alimentaire'!N4</f>
+        <f>'Op. Agro-alimentaire'!B13</f>
         <v/>
       </c>
       <c r="D5" s="10">
-        <f>'Op. Agro-alimentaire'!N6</f>
+        <f>'Op. Agro-alimentaire'!B14</f>
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>'Op. Agro-alimentaire'!N8</f>
+        <f>'Op. Agro-alimentaire'!B15</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>'Op. Agro-alimentaire'!N10</f>
+        <f>'Op. Agro-alimentaire'!H10</f>
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>'Op. Agro-alimentaire'!N12</f>
+        <f>'Op. Agro-alimentaire'!I10</f>
         <v/>
       </c>
       <c r="H5" s="11">
-        <f>'Op. Agro-alimentaire'!N13</f>
+        <f>'Op. Agro-alimentaire'!J10</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="12" t="inlineStr"/>
+      <c r="A6" s="12" t="n"/>
       <c r="B6" s="13" t="inlineStr">
         <is>
           <t>TOTAL</t>
@@ -793,7 +781,7 @@
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>Pour ajouter une nouvelle opération : créer une feuille sur le modèle "Op. Agro-alimentaire" et ajouter une ligne dans ce tableau.</t>
+          <t>Pour ajouter une opération : créer une nouvelle feuille et ajouter une ligne dans ce tableau.</t>
         </is>
       </c>
     </row>
@@ -813,17 +801,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="0.5" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -879,10 +866,6 @@
       <c r="E4" s="9" t="n"/>
       <c r="F4" s="9" t="n"/>
       <c r="G4" s="9" t="n"/>
-      <c r="N4" s="21">
-        <f>B3</f>
-        <v/>
-      </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -914,10 +897,6 @@
       <c r="E6" s="9" t="n"/>
       <c r="F6" s="9" t="n"/>
       <c r="G6" s="9" t="n"/>
-      <c r="N6" s="21">
-        <f>B4</f>
-        <v/>
-      </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -935,40 +914,36 @@
       <c r="G7" s="5" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>Bénéfice Net Total</t>
         </is>
       </c>
-      <c r="B8" s="23">
+      <c r="B8" s="22">
         <f>B6+B7</f>
         <v/>
       </c>
-      <c r="C8" s="24" t="n"/>
-      <c r="D8" s="24" t="n"/>
-      <c r="E8" s="24" t="n"/>
-      <c r="F8" s="24" t="n"/>
-      <c r="G8" s="24" t="n"/>
-      <c r="N8" s="21">
-        <f>B5</f>
-        <v/>
-      </c>
+      <c r="C8" s="23" t="n"/>
+      <c r="D8" s="23" t="n"/>
+      <c r="E8" s="23" t="n"/>
+      <c r="F8" s="23" t="n"/>
+      <c r="G8" s="23" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Chiffre d'Affaires</t>
         </is>
       </c>
-      <c r="B9" s="23">
+      <c r="B9" s="22">
         <f>B4+B8</f>
         <v/>
       </c>
-      <c r="C9" s="24" t="n"/>
-      <c r="D9" s="24" t="n"/>
-      <c r="E9" s="24" t="n"/>
-      <c r="F9" s="24" t="n"/>
-      <c r="G9" s="24" t="n"/>
+      <c r="C9" s="23" t="n"/>
+      <c r="D9" s="23" t="n"/>
+      <c r="E9" s="23" t="n"/>
+      <c r="F9" s="23" t="n"/>
+      <c r="G9" s="23" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
@@ -985,24 +960,8 @@
       <c r="E10" s="9" t="n"/>
       <c r="F10" s="9" t="n"/>
       <c r="G10" s="9" t="n"/>
-      <c r="N10" s="21">
-        <f>B9</f>
-        <v/>
-      </c>
     </row>
     <row r="11" ht="22" customHeight="1"/>
-    <row r="12">
-      <c r="N12" s="21">
-        <f>B8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="N13" s="25">
-        <f>B10</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
@@ -1017,7 +976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1027,11 +986,10 @@
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="0.5" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1111,7 +1069,7 @@
           <t>Cobra</t>
         </is>
       </c>
-      <c r="C4" s="26" t="n">
+      <c r="C4" s="24" t="n">
         <v>8</v>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -1141,9 +1099,6 @@
         <f>I4/H4</f>
         <v/>
       </c>
-      <c r="N4" s="21" t="n">
-        <v>500000</v>
-      </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
@@ -1156,7 +1111,7 @@
           <t>Ndiamb</t>
         </is>
       </c>
-      <c r="C5" s="27" t="n">
+      <c r="C5" s="25" t="n">
         <v>4</v>
       </c>
       <c r="D5" s="8" t="inlineStr">
@@ -1198,7 +1153,7 @@
           <t>Sofia</t>
         </is>
       </c>
-      <c r="C6" s="26" t="n">
+      <c r="C6" s="24" t="n">
         <v>28</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -1228,10 +1183,6 @@
         <f>I6/H6</f>
         <v/>
       </c>
-      <c r="N6" s="21">
-        <f>F10</f>
-        <v/>
-      </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
@@ -1244,7 +1195,7 @@
           <t>Jukuli</t>
         </is>
       </c>
-      <c r="C7" s="27" t="n">
+      <c r="C7" s="25" t="n">
         <v>24</v>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -1286,7 +1237,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C8" s="26" t="n">
+      <c r="C8" s="24" t="n">
         <v>50</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1316,13 +1267,9 @@
         <f>I8/H8</f>
         <v/>
       </c>
-      <c r="N8" s="21">
-        <f>N4-N6</f>
-        <v/>
-      </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="28" t="inlineStr">
+      <c r="A9" s="26" t="inlineStr">
         <is>
           <t>Transport</t>
         </is>
@@ -1331,7 +1278,7 @@
       <c r="C9" s="9" t="n"/>
       <c r="D9" s="9" t="n"/>
       <c r="E9" s="9" t="n"/>
-      <c r="F9" s="29" t="n">
+      <c r="F9" s="27" t="n">
         <v>40000</v>
       </c>
       <c r="G9" s="9" t="n"/>
@@ -1345,15 +1292,15 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B10" s="12" t="n"/>
-      <c r="C10" s="12" t="n"/>
-      <c r="D10" s="12" t="n"/>
-      <c r="E10" s="12" t="n"/>
+      <c r="B10" s="28" t="n"/>
+      <c r="C10" s="28" t="n"/>
+      <c r="D10" s="28" t="n"/>
+      <c r="E10" s="28" t="n"/>
       <c r="F10" s="14">
         <f>SUM(F4:F8)+F9</f>
         <v/>
       </c>
-      <c r="G10" s="12" t="n"/>
+      <c r="G10" s="28" t="n"/>
       <c r="H10" s="14">
         <f>SUM(H4:H8)</f>
         <v/>
@@ -1366,44 +1313,32 @@
         <f>I10/H10</f>
         <v/>
       </c>
-      <c r="N10" s="21">
-        <f>H10</f>
-        <v/>
-      </c>
     </row>
     <row r="11" ht="22" customHeight="1"/>
     <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>BILAN DE L'OPÉRATION</t>
         </is>
       </c>
-      <c r="N12" s="21">
-        <f>I10</f>
-        <v/>
-      </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="24" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>Capital Disponible</t>
         </is>
       </c>
-      <c r="B13" s="31" t="n">
+      <c r="B13" s="29" t="n">
         <v>500000</v>
       </c>
-      <c r="C13" s="24" t="n"/>
-      <c r="D13" s="24" t="n"/>
-      <c r="E13" s="24" t="n"/>
-      <c r="F13" s="24" t="n"/>
-      <c r="G13" s="24" t="n"/>
-      <c r="H13" s="24" t="n"/>
-      <c r="I13" s="24" t="n"/>
-      <c r="J13" s="24" t="n"/>
-      <c r="N13" s="25">
-        <f>N12/N10</f>
-        <v/>
-      </c>
+      <c r="C13" s="23" t="n"/>
+      <c r="D13" s="23" t="n"/>
+      <c r="E13" s="23" t="n"/>
+      <c r="F13" s="23" t="n"/>
+      <c r="G13" s="23" t="n"/>
+      <c r="H13" s="23" t="n"/>
+      <c r="I13" s="23" t="n"/>
+      <c r="J13" s="23" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -1411,7 +1346,7 @@
           <t>Capital Investi</t>
         </is>
       </c>
-      <c r="B14" s="32">
+      <c r="B14" s="30">
         <f>F10</f>
         <v/>
       </c>
@@ -1425,23 +1360,23 @@
       <c r="J14" s="5" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="24" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>Capital en Caisse</t>
         </is>
       </c>
-      <c r="B15" s="23">
+      <c r="B15" s="22">
         <f>B13-B14</f>
         <v/>
       </c>
-      <c r="C15" s="24" t="n"/>
-      <c r="D15" s="24" t="n"/>
-      <c r="E15" s="24" t="n"/>
-      <c r="F15" s="24" t="n"/>
-      <c r="G15" s="24" t="n"/>
-      <c r="H15" s="24" t="n"/>
-      <c r="I15" s="24" t="n"/>
-      <c r="J15" s="24" t="n"/>
+      <c r="C15" s="23" t="n"/>
+      <c r="D15" s="23" t="n"/>
+      <c r="E15" s="23" t="n"/>
+      <c r="F15" s="23" t="n"/>
+      <c r="G15" s="23" t="n"/>
+      <c r="H15" s="23" t="n"/>
+      <c r="I15" s="23" t="n"/>
+      <c r="J15" s="23" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
@@ -1449,7 +1384,7 @@
           <t>Chiffre d'Affaires</t>
         </is>
       </c>
-      <c r="B16" s="32">
+      <c r="B16" s="30">
         <f>H10</f>
         <v/>
       </c>
@@ -1463,23 +1398,23 @@
       <c r="J16" s="5" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="24" t="inlineStr">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t>Bénéfice Net</t>
         </is>
       </c>
-      <c r="B17" s="23">
+      <c r="B17" s="22">
         <f>I10</f>
         <v/>
       </c>
-      <c r="C17" s="24" t="n"/>
-      <c r="D17" s="24" t="n"/>
-      <c r="E17" s="24" t="n"/>
-      <c r="F17" s="24" t="n"/>
-      <c r="G17" s="24" t="n"/>
-      <c r="H17" s="24" t="n"/>
-      <c r="I17" s="24" t="n"/>
-      <c r="J17" s="24" t="n"/>
+      <c r="C17" s="23" t="n"/>
+      <c r="D17" s="23" t="n"/>
+      <c r="E17" s="23" t="n"/>
+      <c r="F17" s="23" t="n"/>
+      <c r="G17" s="23" t="n"/>
+      <c r="H17" s="23" t="n"/>
+      <c r="I17" s="23" t="n"/>
+      <c r="J17" s="23" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -1487,7 +1422,7 @@
           <t>Marge Nette</t>
         </is>
       </c>
-      <c r="B18" s="33">
+      <c r="B18" s="31">
         <f>J10</f>
         <v/>
       </c>

</xml_diff>